<commit_message>
update / fix excel/ hide search data management updating currency/ search - purchaseAnalysis/ category - database
</commit_message>
<xml_diff>
--- a/WpfApp2/excelTemplate/template.xlsx
+++ b/WpfApp2/excelTemplate/template.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12336"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12432"/>
   </bookViews>
   <sheets>
     <sheet name="BOM ALL" sheetId="8" r:id="rId1"/>
@@ -618,10 +618,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
-  <si>
-    <t>BOM OF NX5 BRACKET BENDING</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t xml:space="preserve">STT
 </t>
@@ -710,7 +707,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="&quot;US$&quot;#,##0_);[Red]\(&quot;US$&quot;#,##0\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;US$&quot;#,##0_);[Red]\(&quot;US$&quot;#,##0\)"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -993,7 +990,7 @@
     <xf numFmtId="3" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1008,7 +1005,7 @@
     <xf numFmtId="2" fontId="15" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1020,13 +1017,13 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1038,13 +1035,13 @@
     <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -1432,9 +1429,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="81.75" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>0</v>
-      </c>
+      <c r="A1" s="30"/>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
       <c r="D1" s="30"/>
@@ -1453,29 +1448,29 @@
     </row>
     <row r="2" spans="1:16" ht="81.75" customHeight="1">
       <c r="A2" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="C2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="D2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="E2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="31" t="s">
-        <v>5</v>
-      </c>
       <c r="F2" s="31" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G2" s="33" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H2" s="34"/>
       <c r="I2" s="33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J2" s="34"/>
       <c r="K2" s="33"/>
@@ -1493,30 +1488,30 @@
       <c r="E3" s="32"/>
       <c r="F3" s="32"/>
       <c r="G3" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I3" s="6"/>
       <c r="J3" s="6"/>
       <c r="K3" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="O3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="M3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="O3" s="6" t="s">
+      <c r="P3" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="102.75" customHeight="1">

</xml_diff>